<commit_message>
Refresh inverter ad summary: drop sub-$1 shop entries from runaway list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ewFohDueaqFzwZmB6CQqn
</commit_message>
<xml_diff>
--- a/reports/逆变器广告_SPU_ASIN_9-10月汇总.xlsx
+++ b/reports/逆变器广告_SPU_ASIN_9-10月汇总.xlsx
@@ -2110,31 +2110,6 @@
       </rPr>
       <t xml:space="preserve">AMZ8-CA $796/ACOS 56%</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">；</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AMZ8-US $0/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">无出单</t>
-    </r>
   </si>
   <si>
     <r>
@@ -4101,40 +4076,7 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AMZ5-US $1578/ACOS 50%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">；</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">HK5-US $0/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">无出单</t>
-    </r>
+    <t xml:space="preserve">AMZ5-US $1578/ACOS 50%</t>
   </si>
   <si>
     <t xml:space="preserve">B0CQ4PFGH5</t>
@@ -8914,11 +8856,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="73430352"/>
-        <c:axId val="42852622"/>
+        <c:axId val="36364208"/>
+        <c:axId val="30137669"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="73430352"/>
+        <c:axId val="36364208"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8950,7 +8892,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42852622"/>
+        <c:crossAx val="30137669"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8958,7 +8900,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42852622"/>
+        <c:axId val="30137669"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9000,7 +8942,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73430352"/>
+        <c:crossAx val="36364208"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9353,11 +9295,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="5203119"/>
-        <c:axId val="26351536"/>
+        <c:axId val="78762734"/>
+        <c:axId val="82480798"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="5203119"/>
+        <c:axId val="78762734"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9389,7 +9331,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26351536"/>
+        <c:crossAx val="82480798"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9397,7 +9339,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="26351536"/>
+        <c:axId val="82480798"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9439,7 +9381,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5203119"/>
+        <c:crossAx val="78762734"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>